<commit_message>
Harden backend security settings, unify design tokens, and polish UI for May UAT release
- Backend: env-driven security headers (HSTS, SSL redirect, X-Frame-Options, clickjacking middleware), .env.local support, deterministic debug secret key
- Frontend: introduce Notion-inspired design token system (type scale, color palette, spacing) in global styles and migrate 30+ component SCSS files
- Refactor my-submissions component (HTML/TS/SCSS) and add compact-submission-card shared component
- Replace proxy.conf.json with proxy.conf.cjs, update Angular/package configs
- Add sprint S06 review/lessons-learned, May 15 UAT handoff doc, Snyk security report
- Add backend .snyk policy and .env.local.example for local dev

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/attached_assets/DMIS_Stakeholder_Personas_v2.2.xlsx
+++ b/docs/attached_assets/DMIS_Stakeholder_Personas_v2.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wbowe\OneDrive\Desktop\project\DMIS_UpdatedVersion\docs\attached_assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1329BCDD-C5C1-4431-B380-4FE8B8D2B85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14BEBEA5-46B2-4357-9984-F47CADAD6692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 Overview" sheetId="1" r:id="rId1"/>
@@ -3887,9 +3887,6 @@
     <t>EP-02 Replenishment (procurement horizon); EP-01 Donations (supplier manifests); EP-08 Cash &amp; Funds; EP-11 Audit</t>
   </si>
   <si>
-    <t>Initiate purchase orders from approved Needs Lists; track supplier delivery timelines; receive and verify GRN against PO; attach supporting documentation; escalate clearance-blocked deliveries; reconcile with Finance Officer.</t>
-  </si>
-  <si>
     <t>GOJ procurement compliance complexity; emergency threshold management (J$3M / J$60M / J$100M tiers); documentation backlogs during surge; clearance bottlenecks for regulated goods; audit pressure.</t>
   </si>
   <si>
@@ -5628,6 +5625,9 @@
   </si>
   <si>
     <t>Appended to DELIVERY section; cross-feed health stewardship and stale-data escalation</t>
+  </si>
+  <si>
+    <t>Initiate request for quotations, purchase orders from approved Needs Lists; track supplier delivery timelines; receive and verify GRN against PO; attach supporting documentation; escalate clearance-blocked deliveries; reconcile with Finance Officer.</t>
   </si>
 </sst>
 </file>
@@ -6302,49 +6302,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6354,6 +6331,65 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6400,42 +6436,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6750,7 +6750,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="97" t="s">
+      <c r="B1" s="107" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="96"/>
@@ -6758,7 +6758,7 @@
       <c r="E1" s="96"/>
     </row>
     <row r="2" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="98" t="s">
+      <c r="B2" s="108" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="96"/>
@@ -6832,7 +6832,7 @@
     </row>
     <row r="12" spans="1:5" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="95" t="s">
+      <c r="B13" s="106" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="96"/>
@@ -7023,8 +7023,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1457</v>
+      <c r="A1" s="97" t="s">
+        <v>1456</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -7043,7 +7043,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="132" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -7117,7 +7117,7 @@
     </row>
     <row r="4" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="61" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>49</v>
@@ -7129,22 +7129,22 @@
         <v>444</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>1458</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>1459</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>1460</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>1461</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>1462</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>1463</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>1464</v>
       </c>
       <c r="K4" s="45" t="s">
         <v>931</v>
@@ -7162,7 +7162,7 @@
         <v>109</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="Q4" s="70" t="s">
         <v>76</v>
@@ -7170,7 +7170,7 @@
     </row>
     <row r="5" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="62" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>49</v>
@@ -7182,22 +7182,22 @@
         <v>452</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>1466</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>1467</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>1468</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>1469</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>1470</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>1471</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>1472</v>
       </c>
       <c r="K5" s="47" t="s">
         <v>931</v>
@@ -7215,7 +7215,7 @@
         <v>109</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
       <c r="Q5" s="70" t="s">
         <v>76</v>
@@ -7223,7 +7223,7 @@
     </row>
     <row r="6" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="61" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>49</v>
@@ -7235,22 +7235,22 @@
         <v>460</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>1474</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>1475</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>1476</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>765</v>
       </c>
       <c r="H6" s="6" t="s">
+        <v>1476</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>1477</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>1478</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>1479</v>
       </c>
       <c r="K6" s="45" t="s">
         <v>931</v>
@@ -7268,7 +7268,7 @@
         <v>82</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1480</v>
+        <v>1479</v>
       </c>
       <c r="Q6" s="70" t="s">
         <v>76</v>
@@ -7276,7 +7276,7 @@
     </row>
     <row r="7" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="62" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>49</v>
@@ -7285,25 +7285,25 @@
         <v>443</v>
       </c>
       <c r="D7" s="8" t="s">
+        <v>1481</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>1482</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>1483</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>1484</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>785</v>
       </c>
       <c r="H7" s="8" t="s">
+        <v>1484</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>1485</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>1486</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>1487</v>
       </c>
       <c r="K7" s="47" t="s">
         <v>931</v>
@@ -7321,7 +7321,7 @@
         <v>109</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
       <c r="Q7" s="70" t="s">
         <v>76</v>
@@ -7329,7 +7329,7 @@
     </row>
     <row r="8" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="61" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>49</v>
@@ -7338,25 +7338,25 @@
         <v>49</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>1489</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>1490</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>1491</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>1492</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>1493</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>1494</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>1495</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>1496</v>
       </c>
       <c r="K8" s="45" t="s">
         <v>900</v>
@@ -7374,7 +7374,7 @@
         <v>109</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>1497</v>
+        <v>1496</v>
       </c>
       <c r="Q8" s="70" t="s">
         <v>76</v>
@@ -7382,7 +7382,7 @@
     </row>
     <row r="9" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="62" t="s">
-        <v>1498</v>
+        <v>1497</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>49</v>
@@ -7394,22 +7394,22 @@
         <v>492</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>1498</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>1499</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>1500</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>1501</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="8" t="s">
         <v>1502</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>1503</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>1504</v>
       </c>
       <c r="K9" s="47" t="s">
         <v>931</v>
@@ -7427,7 +7427,7 @@
         <v>109</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>1505</v>
+        <v>1504</v>
       </c>
       <c r="Q9" s="70" t="s">
         <v>76</v>
@@ -7435,7 +7435,7 @@
     </row>
     <row r="10" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="61" t="s">
-        <v>1506</v>
+        <v>1505</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>49</v>
@@ -7444,25 +7444,25 @@
         <v>443</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>1506</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>1507</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>1508</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>1509</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>791</v>
       </c>
       <c r="H10" s="6" t="s">
+        <v>1509</v>
+      </c>
+      <c r="I10" s="6" t="s">
         <v>1510</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>1511</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>1512</v>
       </c>
       <c r="K10" s="45" t="s">
         <v>931</v>
@@ -7480,7 +7480,7 @@
         <v>82</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>1513</v>
+        <v>1512</v>
       </c>
       <c r="Q10" s="70" t="s">
         <v>76</v>
@@ -7488,7 +7488,7 @@
     </row>
     <row r="11" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="62" t="s">
-        <v>1514</v>
+        <v>1513</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>49</v>
@@ -7497,25 +7497,25 @@
         <v>816</v>
       </c>
       <c r="D11" s="8" t="s">
+        <v>1514</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>1515</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="F11" s="8" t="s">
         <v>1516</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>1517</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>818</v>
       </c>
       <c r="H11" s="8" t="s">
+        <v>1517</v>
+      </c>
+      <c r="I11" s="8" t="s">
         <v>1518</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="J11" s="8" t="s">
         <v>1519</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>1520</v>
       </c>
       <c r="K11" s="47" t="s">
         <v>875</v>
@@ -7533,7 +7533,7 @@
         <v>82</v>
       </c>
       <c r="P11" s="8" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="Q11" s="70" t="s">
         <v>76</v>
@@ -7541,7 +7541,7 @@
     </row>
     <row r="12" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="83" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>49</v>
@@ -7553,22 +7553,22 @@
         <v>624</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>1522</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>1523</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="G12" s="6" t="s">
         <v>1524</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>1525</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>1526</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="J12" s="6" t="s">
         <v>1527</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>1528</v>
       </c>
       <c r="K12" s="6" t="s">
         <v>931</v>
@@ -7586,7 +7586,7 @@
         <v>82</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>1529</v>
+        <v>1528</v>
       </c>
       <c r="Q12" s="70" t="s">
         <v>76</v>
@@ -7621,8 +7621,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1530</v>
+      <c r="A1" s="97" t="s">
+        <v>1529</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -7641,7 +7641,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="121" t="s">
+      <c r="A2" s="133" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -7715,7 +7715,7 @@
     </row>
     <row r="4" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="64" t="s">
-        <v>1531</v>
+        <v>1530</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>52</v>
@@ -7727,22 +7727,22 @@
         <v>503</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>1531</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>1532</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>1533</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>1534</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>1535</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>1536</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>1537</v>
       </c>
       <c r="K4" s="45" t="s">
         <v>931</v>
@@ -7760,7 +7760,7 @@
         <v>109</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1538</v>
+        <v>1537</v>
       </c>
       <c r="Q4" s="71" t="s">
         <v>227</v>
@@ -7768,7 +7768,7 @@
     </row>
     <row r="5" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="65" t="s">
-        <v>1539</v>
+        <v>1538</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>52</v>
@@ -7780,22 +7780,22 @@
         <v>511</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>1539</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>1540</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>1541</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>1542</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>1543</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>1544</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>1545</v>
       </c>
       <c r="K5" s="47" t="s">
         <v>931</v>
@@ -7813,7 +7813,7 @@
         <v>109</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>1546</v>
+        <v>1545</v>
       </c>
       <c r="Q5" s="71" t="s">
         <v>227</v>
@@ -7821,7 +7821,7 @@
     </row>
     <row r="6" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="64" t="s">
-        <v>1547</v>
+        <v>1546</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>52</v>
@@ -7833,22 +7833,22 @@
         <v>519</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>1547</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>1548</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>1549</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>1550</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>1551</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>1552</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>1553</v>
       </c>
       <c r="K6" s="45" t="s">
         <v>931</v>
@@ -7866,7 +7866,7 @@
         <v>109</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1554</v>
+        <v>1553</v>
       </c>
       <c r="Q6" s="71" t="s">
         <v>227</v>
@@ -7874,7 +7874,7 @@
     </row>
     <row r="7" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="65" t="s">
-        <v>1555</v>
+        <v>1554</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>52</v>
@@ -7886,22 +7886,22 @@
         <v>527</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>1555</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>1556</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>1557</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>1558</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>1559</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>1560</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>1561</v>
       </c>
       <c r="K7" s="47" t="s">
         <v>931</v>
@@ -7919,7 +7919,7 @@
         <v>109</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="Q7" s="71" t="s">
         <v>227</v>
@@ -7927,7 +7927,7 @@
     </row>
     <row r="8" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="64" t="s">
-        <v>1563</v>
+        <v>1562</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>52</v>
@@ -7936,25 +7936,25 @@
         <v>502</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>1563</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>1564</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>1565</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>1566</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>1567</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>1568</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>1569</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>1570</v>
       </c>
       <c r="K8" s="45" t="s">
         <v>931</v>
@@ -7972,7 +7972,7 @@
         <v>109</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>1571</v>
+        <v>1570</v>
       </c>
       <c r="Q8" s="71" t="s">
         <v>227</v>
@@ -7980,7 +7980,7 @@
     </row>
     <row r="9" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="65" t="s">
-        <v>1572</v>
+        <v>1571</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>52</v>
@@ -7992,22 +7992,22 @@
         <v>543</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>1572</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>1573</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>1574</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>805</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>1574</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>1575</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>1576</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>1577</v>
       </c>
       <c r="K9" s="47" t="s">
         <v>931</v>
@@ -8025,7 +8025,7 @@
         <v>109</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>1578</v>
+        <v>1577</v>
       </c>
       <c r="Q9" s="71" t="s">
         <v>227</v>
@@ -8033,7 +8033,7 @@
     </row>
     <row r="10" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="64" t="s">
-        <v>1579</v>
+        <v>1578</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>52</v>
@@ -8045,22 +8045,22 @@
         <v>551</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>1579</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>1580</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>1581</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>1582</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>1583</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>1584</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>1585</v>
       </c>
       <c r="K10" s="45" t="s">
         <v>931</v>
@@ -8078,7 +8078,7 @@
         <v>109</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>1586</v>
+        <v>1585</v>
       </c>
       <c r="Q10" s="71" t="s">
         <v>227</v>
@@ -8086,7 +8086,7 @@
     </row>
     <row r="11" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="65" t="s">
-        <v>1587</v>
+        <v>1586</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>52</v>
@@ -8098,22 +8098,22 @@
         <v>559</v>
       </c>
       <c r="E11" s="8" t="s">
+        <v>1587</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>1588</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="G11" s="8" t="s">
         <v>1589</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="H11" s="8" t="s">
         <v>1590</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="I11" s="8" t="s">
         <v>1591</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="J11" s="8" t="s">
         <v>1592</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>1593</v>
       </c>
       <c r="K11" s="47" t="s">
         <v>931</v>
@@ -8131,7 +8131,7 @@
         <v>109</v>
       </c>
       <c r="P11" s="8" t="s">
-        <v>1594</v>
+        <v>1593</v>
       </c>
       <c r="Q11" s="71" t="s">
         <v>227</v>
@@ -8139,7 +8139,7 @@
     </row>
     <row r="12" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="64" t="s">
-        <v>1595</v>
+        <v>1594</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>52</v>
@@ -8151,22 +8151,22 @@
         <v>580</v>
       </c>
       <c r="E12" s="6" t="s">
+        <v>1595</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>1596</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>1597</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>811</v>
       </c>
       <c r="H12" s="6" t="s">
+        <v>1597</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>1598</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="J12" s="6" t="s">
         <v>1599</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>1600</v>
       </c>
       <c r="K12" s="45" t="s">
         <v>931</v>
@@ -8184,7 +8184,7 @@
         <v>109</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>1601</v>
+        <v>1600</v>
       </c>
       <c r="Q12" s="71" t="s">
         <v>227</v>
@@ -8192,7 +8192,7 @@
     </row>
     <row r="13" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="65" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>52</v>
@@ -8201,25 +8201,25 @@
         <v>579</v>
       </c>
       <c r="D13" s="8" t="s">
+        <v>1602</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>1603</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="F13" s="8" t="s">
         <v>1604</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>1605</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>815</v>
       </c>
       <c r="H13" s="8" t="s">
+        <v>1605</v>
+      </c>
+      <c r="I13" s="8" t="s">
         <v>1606</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="J13" s="8" t="s">
         <v>1607</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>1608</v>
       </c>
       <c r="K13" s="47" t="s">
         <v>931</v>
@@ -8237,7 +8237,7 @@
         <v>109</v>
       </c>
       <c r="P13" s="8" t="s">
-        <v>1609</v>
+        <v>1608</v>
       </c>
       <c r="Q13" s="71" t="s">
         <v>227</v>
@@ -8245,34 +8245,34 @@
     </row>
     <row r="14" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="84" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>52</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>568</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>1611</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>1612</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>1613</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>1614</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>1615</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="J14" s="6" t="s">
         <v>1616</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>1617</v>
       </c>
       <c r="K14" s="6" t="s">
         <v>931</v>
@@ -8290,7 +8290,7 @@
         <v>109</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>1618</v>
+        <v>1617</v>
       </c>
       <c r="Q14" s="71" t="s">
         <v>227</v>
@@ -8325,8 +8325,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1619</v>
+      <c r="A1" s="97" t="s">
+        <v>1618</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -8345,7 +8345,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="122" t="s">
+      <c r="A2" s="134" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -8419,7 +8419,7 @@
     </row>
     <row r="4" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="67" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>55</v>
@@ -8431,22 +8431,22 @@
         <v>655</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>1620</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>1621</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>1622</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>825</v>
       </c>
       <c r="H4" s="6" t="s">
+        <v>1622</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>1623</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>1624</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>1625</v>
       </c>
       <c r="K4" s="45" t="s">
         <v>854</v>
@@ -8464,7 +8464,7 @@
         <v>82</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1626</v>
+        <v>1625</v>
       </c>
       <c r="Q4" s="70" t="s">
         <v>76</v>
@@ -8472,7 +8472,7 @@
     </row>
     <row r="5" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="68" t="s">
-        <v>1627</v>
+        <v>1626</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>55</v>
@@ -8484,22 +8484,22 @@
         <v>663</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>1627</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>1628</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>1629</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>826</v>
       </c>
       <c r="H5" s="8" t="s">
+        <v>1629</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>1630</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>1631</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>1632</v>
       </c>
       <c r="K5" s="47" t="s">
         <v>854</v>
@@ -8517,7 +8517,7 @@
         <v>82</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>1633</v>
+        <v>1632</v>
       </c>
       <c r="Q5" s="70" t="s">
         <v>76</v>
@@ -8525,7 +8525,7 @@
     </row>
     <row r="6" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="67" t="s">
-        <v>1634</v>
+        <v>1633</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>55</v>
@@ -8537,22 +8537,22 @@
         <v>671</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>1634</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>1635</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>1636</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>827</v>
       </c>
       <c r="H6" s="6" t="s">
+        <v>1636</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>1637</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>1638</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>1639</v>
       </c>
       <c r="K6" s="45" t="s">
         <v>854</v>
@@ -8570,7 +8570,7 @@
         <v>109</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="Q6" s="70" t="s">
         <v>76</v>
@@ -8578,7 +8578,7 @@
     </row>
     <row r="7" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="68" t="s">
-        <v>1641</v>
+        <v>1640</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>55</v>
@@ -8590,22 +8590,22 @@
         <v>679</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>1641</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>1642</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>1643</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>828</v>
       </c>
       <c r="H7" s="8" t="s">
+        <v>1643</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>1644</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>1645</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>1646</v>
       </c>
       <c r="K7" s="47" t="s">
         <v>875</v>
@@ -8623,7 +8623,7 @@
         <v>109</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>1647</v>
+        <v>1646</v>
       </c>
       <c r="Q7" s="70" t="s">
         <v>76</v>
@@ -8631,7 +8631,7 @@
     </row>
     <row r="8" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="67" t="s">
-        <v>1648</v>
+        <v>1647</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>55</v>
@@ -8643,22 +8643,22 @@
         <v>687</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>1648</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>1649</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>1650</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>829</v>
       </c>
       <c r="H8" s="6" t="s">
+        <v>1650</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>1651</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>1652</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>1653</v>
       </c>
       <c r="K8" s="45" t="s">
         <v>854</v>
@@ -8676,7 +8676,7 @@
         <v>109</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="Q8" s="70" t="s">
         <v>76</v>
@@ -8684,10 +8684,10 @@
     </row>
     <row r="9" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="85" t="s">
+        <v>1654</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>1655</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>1656</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>654</v>
@@ -8696,22 +8696,22 @@
         <v>695</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>1656</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>1657</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>1658</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>1659</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="8" t="s">
         <v>1660</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>1661</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>1662</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>854</v>
@@ -8729,7 +8729,7 @@
         <v>82</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>1663</v>
+        <v>1662</v>
       </c>
       <c r="Q9" s="70" t="s">
         <v>76</v>
@@ -8737,10 +8737,10 @@
     </row>
     <row r="10" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="86" t="s">
+        <v>1663</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>1664</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>1665</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>703</v>
@@ -8749,22 +8749,22 @@
         <v>704</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>1665</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>1666</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>1667</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>1668</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>1669</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>1670</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>1671</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>864</v>
@@ -8782,7 +8782,7 @@
         <v>109</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="Q10" s="70" t="s">
         <v>76</v>
@@ -8806,8 +8806,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1673</v>
+      <c r="A1" s="97" t="s">
+        <v>1672</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -8861,16 +8861,16 @@
         <v>66</v>
       </c>
       <c r="I3" s="69" t="s">
+        <v>1673</v>
+      </c>
+      <c r="J3" s="69" t="s">
         <v>1674</v>
-      </c>
-      <c r="J3" s="69" t="s">
-        <v>1675</v>
       </c>
       <c r="K3" s="69" t="s">
         <v>847</v>
       </c>
       <c r="L3" s="69" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -8899,16 +8899,16 @@
         <v>82</v>
       </c>
       <c r="I4" s="4" t="s">
+        <v>1676</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>1677</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>1678</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>855</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -8937,10 +8937,10 @@
         <v>109</v>
       </c>
       <c r="I5" s="3" t="s">
+        <v>1679</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>1680</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>1681</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>1001</v>
@@ -8954,7 +8954,7 @@
         <v>40</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>111</v>
@@ -8969,16 +8969,16 @@
         <v>856</v>
       </c>
       <c r="I6" s="4" t="s">
+        <v>1682</v>
+      </c>
+      <c r="J6" s="4" t="s">
         <v>1683</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>1684</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>994</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>1685</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -8986,7 +8986,7 @@
         <v>43</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1686</v>
+        <v>1685</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>101</v>
@@ -8995,16 +8995,16 @@
         <v>880</v>
       </c>
       <c r="I7" s="3" t="s">
+        <v>1686</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>1687</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>1688</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>1689</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -9015,7 +9015,7 @@
         <v>900</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -9026,7 +9026,7 @@
         <v>931</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>1691</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -9034,7 +9034,7 @@
         <v>52</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>1692</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -9044,7 +9044,7 @@
     </row>
     <row r="12" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>1693</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -9078,24 +9078,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="126" t="s">
-        <v>1694</v>
+      <c r="A1" s="138" t="s">
+        <v>1693</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
       <c r="D1" s="96"/>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="124" t="s">
-        <v>1695</v>
+      <c r="A2" s="136" t="s">
+        <v>1694</v>
       </c>
       <c r="B2" s="96"/>
       <c r="C2" s="96"/>
       <c r="D2" s="96"/>
     </row>
     <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="127" t="s">
-        <v>1696</v>
+      <c r="A3" s="139" t="s">
+        <v>1695</v>
       </c>
       <c r="B3" s="96"/>
       <c r="C3" s="96"/>
@@ -9106,10 +9106,10 @@
         <v>1159</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>1696</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>1697</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>1698</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>722</v>
@@ -9120,10 +9120,10 @@
         <v>1276</v>
       </c>
       <c r="B5" s="87" t="s">
+        <v>1698</v>
+      </c>
+      <c r="C5" s="87" t="s">
         <v>1699</v>
-      </c>
-      <c r="C5" s="87" t="s">
-        <v>1700</v>
       </c>
       <c r="D5" s="87" t="s">
         <v>76</v>
@@ -9131,13 +9131,13 @@
     </row>
     <row r="6" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="88" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="B6" s="88" t="s">
+        <v>1700</v>
+      </c>
+      <c r="C6" s="88" t="s">
         <v>1701</v>
-      </c>
-      <c r="C6" s="88" t="s">
-        <v>1702</v>
       </c>
       <c r="D6" s="88" t="s">
         <v>76</v>
@@ -9145,13 +9145,13 @@
     </row>
     <row r="7" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="87" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="B7" s="87" t="s">
+        <v>1702</v>
+      </c>
+      <c r="C7" s="87" t="s">
         <v>1703</v>
-      </c>
-      <c r="C7" s="87" t="s">
-        <v>1704</v>
       </c>
       <c r="D7" s="87" t="s">
         <v>76</v>
@@ -9159,13 +9159,13 @@
     </row>
     <row r="8" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="88" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="B8" s="88" t="s">
         <v>355</v>
       </c>
       <c r="C8" s="88" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="D8" s="88" t="s">
         <v>76</v>
@@ -9173,13 +9173,13 @@
     </row>
     <row r="9" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="87" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="B9" s="87" t="s">
         <v>568</v>
       </c>
       <c r="C9" s="87" t="s">
-        <v>1706</v>
+        <v>1705</v>
       </c>
       <c r="D9" s="87" t="s">
         <v>227</v>
@@ -9187,13 +9187,13 @@
     </row>
     <row r="10" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="88" t="s">
-        <v>1522</v>
+        <v>1521</v>
       </c>
       <c r="B10" s="88" t="s">
         <v>624</v>
       </c>
       <c r="C10" s="88" t="s">
-        <v>1707</v>
+        <v>1706</v>
       </c>
       <c r="D10" s="88" t="s">
         <v>76</v>
@@ -9201,13 +9201,13 @@
     </row>
     <row r="11" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="87" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="B11" s="87" t="s">
+        <v>1707</v>
+      </c>
+      <c r="C11" s="87" t="s">
         <v>1708</v>
-      </c>
-      <c r="C11" s="87" t="s">
-        <v>1709</v>
       </c>
       <c r="D11" s="87" t="s">
         <v>76</v>
@@ -9215,21 +9215,21 @@
     </row>
     <row r="12" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="88" t="s">
-        <v>1664</v>
+        <v>1663</v>
       </c>
       <c r="B12" s="88" t="s">
         <v>704</v>
       </c>
       <c r="C12" s="88" t="s">
+        <v>1709</v>
+      </c>
+      <c r="D12" s="88" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="135" t="s">
         <v>1710</v>
-      </c>
-      <c r="D12" s="88" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="123" t="s">
-        <v>1711</v>
       </c>
       <c r="B13" s="96"/>
       <c r="C13" s="96"/>
@@ -9237,16 +9237,16 @@
     </row>
     <row r="14" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>1711</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>1712</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>1713</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>1714</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>1715</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -9257,10 +9257,10 @@
         <v>117</v>
       </c>
       <c r="C15" s="87" t="s">
+        <v>1715</v>
+      </c>
+      <c r="D15" s="87" t="s">
         <v>1716</v>
-      </c>
-      <c r="D15" s="87" t="s">
-        <v>1717</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -9271,24 +9271,24 @@
         <v>872</v>
       </c>
       <c r="C16" s="88" t="s">
+        <v>1717</v>
+      </c>
+      <c r="D16" s="88" t="s">
         <v>1718</v>
-      </c>
-      <c r="D16" s="88" t="s">
-        <v>1719</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="87" t="s">
-        <v>1720</v>
+        <v>1719</v>
       </c>
       <c r="B17" s="87" t="s">
         <v>126</v>
       </c>
       <c r="C17" s="87" t="s">
+        <v>1720</v>
+      </c>
+      <c r="D17" s="87" t="s">
         <v>1721</v>
-      </c>
-      <c r="D17" s="87" t="s">
-        <v>1722</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -9299,10 +9299,10 @@
         <v>134</v>
       </c>
       <c r="C18" s="88" t="s">
+        <v>1722</v>
+      </c>
+      <c r="D18" s="88" t="s">
         <v>1723</v>
-      </c>
-      <c r="D18" s="88" t="s">
-        <v>1724</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -9313,38 +9313,38 @@
         <v>177</v>
       </c>
       <c r="C19" s="87" t="s">
+        <v>1724</v>
+      </c>
+      <c r="D19" s="87" t="s">
         <v>1725</v>
-      </c>
-      <c r="D19" s="87" t="s">
-        <v>1726</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="88" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="B20" s="88" t="s">
         <v>265</v>
       </c>
       <c r="C20" s="88" t="s">
+        <v>1727</v>
+      </c>
+      <c r="D20" s="88" t="s">
         <v>1728</v>
-      </c>
-      <c r="D20" s="88" t="s">
-        <v>1729</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="87" t="s">
+        <v>1729</v>
+      </c>
+      <c r="B21" s="87" t="s">
         <v>1730</v>
       </c>
-      <c r="B21" s="87" t="s">
+      <c r="C21" s="87" t="s">
         <v>1731</v>
       </c>
-      <c r="C21" s="87" t="s">
+      <c r="D21" s="87" t="s">
         <v>1732</v>
-      </c>
-      <c r="D21" s="87" t="s">
-        <v>1733</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -9352,18 +9352,18 @@
         <v>384</v>
       </c>
       <c r="B22" s="88" t="s">
+        <v>1733</v>
+      </c>
+      <c r="C22" s="88" t="s">
         <v>1734</v>
       </c>
-      <c r="C22" s="88" t="s">
+      <c r="D22" s="88" t="s">
         <v>1735</v>
       </c>
-      <c r="D22" s="88" t="s">
+    </row>
+    <row r="23" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="140" t="s">
         <v>1736</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="128" t="s">
-        <v>1737</v>
       </c>
       <c r="B23" s="96"/>
       <c r="C23" s="96"/>
@@ -9371,91 +9371,91 @@
     </row>
     <row r="24" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>1737</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>1738</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>1739</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>1740</v>
       </c>
       <c r="D24" s="89"/>
     </row>
     <row r="25" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="87" t="s">
+        <v>1740</v>
+      </c>
+      <c r="B25" s="87" t="s">
         <v>1741</v>
       </c>
-      <c r="B25" s="87" t="s">
+      <c r="C25" s="87" t="s">
         <v>1742</v>
-      </c>
-      <c r="C25" s="87" t="s">
-        <v>1743</v>
       </c>
       <c r="D25" s="87"/>
     </row>
     <row r="26" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="88" t="s">
+        <v>1743</v>
+      </c>
+      <c r="B26" s="88" t="s">
         <v>1744</v>
       </c>
-      <c r="B26" s="88" t="s">
+      <c r="C26" s="88" t="s">
         <v>1745</v>
-      </c>
-      <c r="C26" s="88" t="s">
-        <v>1746</v>
       </c>
       <c r="D26" s="88"/>
     </row>
     <row r="27" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="87" t="s">
+        <v>1746</v>
+      </c>
+      <c r="B27" s="87" t="s">
         <v>1747</v>
       </c>
-      <c r="B27" s="87" t="s">
+      <c r="C27" s="87" t="s">
         <v>1748</v>
-      </c>
-      <c r="C27" s="87" t="s">
-        <v>1749</v>
       </c>
       <c r="D27" s="87"/>
     </row>
     <row r="28" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="88" t="s">
+        <v>1749</v>
+      </c>
+      <c r="B28" s="88" t="s">
         <v>1750</v>
       </c>
-      <c r="B28" s="88" t="s">
+      <c r="C28" s="88" t="s">
         <v>1751</v>
-      </c>
-      <c r="C28" s="88" t="s">
-        <v>1752</v>
       </c>
       <c r="D28" s="88"/>
     </row>
     <row r="29" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="87" t="s">
+        <v>1752</v>
+      </c>
+      <c r="B29" s="87" t="s">
         <v>1753</v>
       </c>
-      <c r="B29" s="87" t="s">
+      <c r="C29" s="87" t="s">
         <v>1754</v>
-      </c>
-      <c r="C29" s="87" t="s">
-        <v>1755</v>
       </c>
       <c r="D29" s="87"/>
     </row>
     <row r="30" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="88" t="s">
+        <v>1755</v>
+      </c>
+      <c r="B30" s="88" t="s">
         <v>1756</v>
       </c>
-      <c r="B30" s="88" t="s">
+      <c r="C30" s="88" t="s">
         <v>1757</v>
       </c>
-      <c r="C30" s="88" t="s">
+      <c r="D30" s="88"/>
+    </row>
+    <row r="31" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="141" t="s">
         <v>1758</v>
-      </c>
-      <c r="D30" s="88"/>
-    </row>
-    <row r="31" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="129" t="s">
-        <v>1759</v>
       </c>
       <c r="B31" s="96"/>
       <c r="C31" s="96"/>
@@ -9463,10 +9463,10 @@
     </row>
     <row r="32" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>1759</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>1760</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>1761</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>850</v>
@@ -9475,31 +9475,31 @@
     </row>
     <row r="33" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="87" t="s">
+        <v>1761</v>
+      </c>
+      <c r="B33" s="87" t="s">
         <v>1762</v>
       </c>
-      <c r="B33" s="87" t="s">
+      <c r="C33" s="87" t="s">
         <v>1763</v>
-      </c>
-      <c r="C33" s="87" t="s">
-        <v>1764</v>
       </c>
       <c r="D33" s="87"/>
     </row>
     <row r="34" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="88" t="s">
+        <v>1764</v>
+      </c>
+      <c r="B34" s="88" t="s">
         <v>1765</v>
       </c>
-      <c r="B34" s="88" t="s">
+      <c r="C34" s="88" t="s">
         <v>1766</v>
       </c>
-      <c r="C34" s="88" t="s">
+      <c r="D34" s="88"/>
+    </row>
+    <row r="35" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="137" t="s">
         <v>1767</v>
-      </c>
-      <c r="D34" s="88"/>
-    </row>
-    <row r="35" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="125" t="s">
-        <v>1768</v>
       </c>
       <c r="B35" s="96"/>
       <c r="C35" s="96"/>
@@ -9507,120 +9507,120 @@
     </row>
     <row r="36" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>1768</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>1769</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>1770</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>1771</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>1772</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="87" t="s">
+        <v>1772</v>
+      </c>
+      <c r="B37" s="87" t="s">
         <v>1773</v>
       </c>
-      <c r="B37" s="87" t="s">
+      <c r="C37" s="87" t="s">
         <v>1774</v>
       </c>
-      <c r="C37" s="87" t="s">
+      <c r="D37" s="87" t="s">
         <v>1775</v>
-      </c>
-      <c r="D37" s="87" t="s">
-        <v>1776</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="88" t="s">
+        <v>1776</v>
+      </c>
+      <c r="B38" s="88" t="s">
         <v>1777</v>
       </c>
-      <c r="B38" s="88" t="s">
+      <c r="C38" s="88" t="s">
         <v>1778</v>
       </c>
-      <c r="C38" s="88" t="s">
+      <c r="D38" s="88" t="s">
         <v>1779</v>
-      </c>
-      <c r="D38" s="88" t="s">
-        <v>1780</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="87" t="s">
+        <v>1780</v>
+      </c>
+      <c r="B39" s="87" t="s">
         <v>1781</v>
       </c>
-      <c r="B39" s="87" t="s">
+      <c r="C39" s="87" t="s">
         <v>1782</v>
       </c>
-      <c r="C39" s="87" t="s">
+      <c r="D39" s="87" t="s">
         <v>1783</v>
-      </c>
-      <c r="D39" s="87" t="s">
-        <v>1784</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="88" t="s">
+        <v>1784</v>
+      </c>
+      <c r="B40" s="88" t="s">
         <v>1785</v>
       </c>
-      <c r="B40" s="88" t="s">
+      <c r="C40" s="88" t="s">
         <v>1786</v>
       </c>
-      <c r="C40" s="88" t="s">
+      <c r="D40" s="88" t="s">
         <v>1787</v>
-      </c>
-      <c r="D40" s="88" t="s">
-        <v>1788</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="87" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B41" s="87" t="s">
         <v>1789</v>
       </c>
-      <c r="B41" s="87" t="s">
+      <c r="C41" s="87" t="s">
         <v>1790</v>
       </c>
-      <c r="C41" s="87" t="s">
+      <c r="D41" s="87" t="s">
         <v>1791</v>
-      </c>
-      <c r="D41" s="87" t="s">
-        <v>1792</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="88" t="s">
+        <v>1792</v>
+      </c>
+      <c r="B42" s="88" t="s">
         <v>1793</v>
       </c>
-      <c r="B42" s="88" t="s">
+      <c r="C42" s="88" t="s">
         <v>1794</v>
       </c>
-      <c r="C42" s="88" t="s">
+      <c r="D42" s="88" t="s">
         <v>1795</v>
-      </c>
-      <c r="D42" s="88" t="s">
-        <v>1796</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="87" t="s">
+        <v>1796</v>
+      </c>
+      <c r="B43" s="87" t="s">
         <v>1797</v>
       </c>
-      <c r="B43" s="87" t="s">
+      <c r="C43" s="87" t="s">
         <v>1798</v>
       </c>
-      <c r="C43" s="87" t="s">
+      <c r="D43" s="87" t="s">
         <v>1799</v>
-      </c>
-      <c r="D43" s="87" t="s">
-        <v>1800</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="45" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="127" t="s">
-        <v>1801</v>
+      <c r="A45" s="139" t="s">
+        <v>1800</v>
       </c>
       <c r="B45" s="96"/>
       <c r="C45" s="96"/>
@@ -9628,162 +9628,162 @@
     </row>
     <row r="46" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="69" t="s">
+        <v>1801</v>
+      </c>
+      <c r="B46" s="69" t="s">
         <v>1802</v>
       </c>
-      <c r="B46" s="69" t="s">
+      <c r="C46" s="69" t="s">
         <v>1803</v>
       </c>
-      <c r="C46" s="69" t="s">
-        <v>1804</v>
-      </c>
       <c r="D46" s="69" t="s">
-        <v>1772</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="87" t="s">
+        <v>1804</v>
+      </c>
+      <c r="B47" s="87" t="s">
         <v>1805</v>
       </c>
-      <c r="B47" s="87" t="s">
+      <c r="C47" s="87" t="s">
         <v>1806</v>
       </c>
-      <c r="C47" s="87" t="s">
+      <c r="D47" s="87" t="s">
         <v>1807</v>
-      </c>
-      <c r="D47" s="87" t="s">
-        <v>1808</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="88" t="s">
+        <v>1808</v>
+      </c>
+      <c r="B48" s="88" t="s">
         <v>1809</v>
       </c>
-      <c r="B48" s="88" t="s">
+      <c r="C48" s="88" t="s">
         <v>1810</v>
       </c>
-      <c r="C48" s="88" t="s">
-        <v>1811</v>
-      </c>
       <c r="D48" s="88" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="87" t="s">
+        <v>1811</v>
+      </c>
+      <c r="B49" s="87" t="s">
         <v>1812</v>
       </c>
-      <c r="B49" s="87" t="s">
+      <c r="C49" s="87" t="s">
         <v>1813</v>
       </c>
-      <c r="C49" s="87" t="s">
-        <v>1814</v>
-      </c>
       <c r="D49" s="87" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="88" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B50" s="88" t="s">
         <v>1815</v>
       </c>
-      <c r="B50" s="88" t="s">
+      <c r="C50" s="88" t="s">
         <v>1816</v>
       </c>
-      <c r="C50" s="88" t="s">
-        <v>1817</v>
-      </c>
       <c r="D50" s="88" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="87" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B51" s="87" t="s">
         <v>1818</v>
       </c>
-      <c r="B51" s="87" t="s">
+      <c r="C51" s="87" t="s">
         <v>1819</v>
       </c>
-      <c r="C51" s="87" t="s">
-        <v>1820</v>
-      </c>
       <c r="D51" s="87" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="88" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B52" s="88" t="s">
         <v>1821</v>
       </c>
-      <c r="B52" s="88" t="s">
+      <c r="C52" s="88" t="s">
         <v>1822</v>
       </c>
-      <c r="C52" s="88" t="s">
-        <v>1823</v>
-      </c>
       <c r="D52" s="88" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="87" t="s">
+        <v>1823</v>
+      </c>
+      <c r="B53" s="87" t="s">
         <v>1824</v>
       </c>
-      <c r="B53" s="87" t="s">
+      <c r="C53" s="87" t="s">
         <v>1825</v>
       </c>
-      <c r="C53" s="87" t="s">
-        <v>1826</v>
-      </c>
       <c r="D53" s="87" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="88" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B54" s="88" t="s">
         <v>1827</v>
       </c>
-      <c r="B54" s="88" t="s">
+      <c r="C54" s="88" t="s">
         <v>1828</v>
       </c>
-      <c r="C54" s="88" t="s">
-        <v>1829</v>
-      </c>
       <c r="D54" s="88" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="87" t="s">
+        <v>1829</v>
+      </c>
+      <c r="B55" s="87" t="s">
         <v>1830</v>
       </c>
-      <c r="B55" s="87" t="s">
+      <c r="C55" s="87" t="s">
         <v>1831</v>
       </c>
-      <c r="C55" s="87" t="s">
-        <v>1832</v>
-      </c>
       <c r="D55" s="87" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="88" t="s">
+        <v>1832</v>
+      </c>
+      <c r="B56" s="88" t="s">
         <v>1833</v>
       </c>
-      <c r="B56" s="88" t="s">
+      <c r="C56" s="88" t="s">
         <v>1834</v>
       </c>
-      <c r="C56" s="88" t="s">
-        <v>1835</v>
-      </c>
       <c r="D56" s="88" t="s">
-        <v>1808</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="59" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="123" t="s">
-        <v>1836</v>
+      <c r="A59" s="135" t="s">
+        <v>1835</v>
       </c>
       <c r="B59" s="96"/>
       <c r="C59" s="96"/>
@@ -9791,16 +9791,16 @@
     </row>
     <row r="60" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="69" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B60" s="69" t="s">
         <v>1837</v>
-      </c>
-      <c r="B60" s="69" t="s">
-        <v>1838</v>
       </c>
       <c r="C60" s="69" t="s">
         <v>1159</v>
       </c>
       <c r="D60" s="69" t="s">
-        <v>1839</v>
+        <v>1838</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9808,13 +9808,13 @@
         <v>695</v>
       </c>
       <c r="B61" s="87" t="s">
+        <v>1839</v>
+      </c>
+      <c r="C61" s="87" t="s">
+        <v>1654</v>
+      </c>
+      <c r="D61" s="87" t="s">
         <v>1840</v>
-      </c>
-      <c r="C61" s="87" t="s">
-        <v>1655</v>
-      </c>
-      <c r="D61" s="87" t="s">
-        <v>1841</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9822,33 +9822,33 @@
         <v>134</v>
       </c>
       <c r="B62" s="88" t="s">
-        <v>1842</v>
+        <v>1841</v>
       </c>
       <c r="C62" s="88" t="s">
         <v>1224</v>
       </c>
       <c r="D62" s="88" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="87" t="s">
+        <v>1843</v>
+      </c>
+      <c r="B63" s="87" t="s">
         <v>1844</v>
       </c>
-      <c r="B63" s="87" t="s">
+      <c r="C63" s="87" t="s">
         <v>1845</v>
       </c>
-      <c r="C63" s="87" t="s">
+      <c r="D63" s="87" t="s">
         <v>1846</v>
-      </c>
-      <c r="D63" s="87" t="s">
-        <v>1847</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="125" t="s">
-        <v>1848</v>
+      <c r="A66" s="137" t="s">
+        <v>1847</v>
       </c>
       <c r="B66" s="96"/>
       <c r="C66" s="96"/>
@@ -9856,16 +9856,16 @@
     </row>
     <row r="67" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="69" t="s">
+        <v>1848</v>
+      </c>
+      <c r="B67" s="69" t="s">
         <v>1849</v>
       </c>
-      <c r="B67" s="69" t="s">
+      <c r="C67" s="69" t="s">
         <v>1850</v>
       </c>
-      <c r="C67" s="69" t="s">
+      <c r="D67" s="69" t="s">
         <v>1851</v>
-      </c>
-      <c r="D67" s="69" t="s">
-        <v>1852</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9879,7 +9879,7 @@
         <v>76</v>
       </c>
       <c r="D68" s="88" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9893,7 +9893,7 @@
         <v>76</v>
       </c>
       <c r="D69" s="87" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9907,7 +9907,7 @@
         <v>76</v>
       </c>
       <c r="D70" s="88" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9921,7 +9921,7 @@
         <v>76</v>
       </c>
       <c r="D71" s="87" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9935,7 +9935,7 @@
         <v>227</v>
       </c>
       <c r="D72" s="88" t="s">
-        <v>1857</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9949,7 +9949,7 @@
         <v>76</v>
       </c>
       <c r="D73" s="87" t="s">
-        <v>1858</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="74" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9963,7 +9963,7 @@
         <v>76</v>
       </c>
       <c r="D74" s="88" t="s">
-        <v>1859</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -9977,7 +9977,7 @@
         <v>76</v>
       </c>
       <c r="D75" s="87" t="s">
-        <v>1860</v>
+        <v>1859</v>
       </c>
     </row>
   </sheetData>
@@ -10015,7 +10015,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="97" t="s">
         <v>59</v>
       </c>
       <c r="B1" s="96"/>
@@ -10032,7 +10032,7 @@
       <c r="M1" s="96"/>
     </row>
     <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="109" t="s">
+      <c r="A2" s="120" t="s">
         <v>60</v>
       </c>
       <c r="B2" s="96"/>
@@ -10093,7 +10093,7 @@
       </c>
     </row>
     <row r="4" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="104" t="s">
+      <c r="A4" s="102" t="s">
         <v>75</v>
       </c>
       <c r="B4" s="96"/>
@@ -11257,21 +11257,21 @@
       </c>
     </row>
     <row r="31" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="130" t="s">
+      <c r="A31" s="121" t="s">
         <v>309</v>
       </c>
-      <c r="B31" s="130"/>
-      <c r="C31" s="130"/>
-      <c r="D31" s="130"/>
-      <c r="E31" s="130"/>
-      <c r="F31" s="130"/>
-      <c r="G31" s="130"/>
-      <c r="H31" s="130"/>
-      <c r="I31" s="130"/>
-      <c r="J31" s="130"/>
-      <c r="K31" s="130"/>
-      <c r="L31" s="130"/>
-      <c r="M31" s="131"/>
+      <c r="B31" s="121"/>
+      <c r="C31" s="121"/>
+      <c r="D31" s="121"/>
+      <c r="E31" s="121"/>
+      <c r="F31" s="121"/>
+      <c r="G31" s="121"/>
+      <c r="H31" s="121"/>
+      <c r="I31" s="121"/>
+      <c r="J31" s="121"/>
+      <c r="K31" s="121"/>
+      <c r="L31" s="121"/>
+      <c r="M31" s="122"/>
       <c r="N31" s="70" t="s">
         <v>76</v>
       </c>
@@ -11409,21 +11409,21 @@
       </c>
     </row>
     <row r="35" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="103" t="s">
+      <c r="A35" s="118" t="s">
         <v>310</v>
       </c>
-      <c r="B35" s="99"/>
-      <c r="C35" s="99"/>
-      <c r="D35" s="99"/>
-      <c r="E35" s="99"/>
-      <c r="F35" s="99"/>
-      <c r="G35" s="99"/>
-      <c r="H35" s="99"/>
-      <c r="I35" s="99"/>
-      <c r="J35" s="99"/>
-      <c r="K35" s="99"/>
-      <c r="L35" s="99"/>
-      <c r="M35" s="100"/>
+      <c r="B35" s="116"/>
+      <c r="C35" s="116"/>
+      <c r="D35" s="116"/>
+      <c r="E35" s="116"/>
+      <c r="F35" s="116"/>
+      <c r="G35" s="116"/>
+      <c r="H35" s="116"/>
+      <c r="I35" s="116"/>
+      <c r="J35" s="116"/>
+      <c r="K35" s="116"/>
+      <c r="L35" s="116"/>
+      <c r="M35" s="117"/>
       <c r="N35" s="70" t="s">
         <v>76</v>
       </c>
@@ -11561,7 +11561,7 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="106" t="s">
+      <c r="A39" s="101" t="s">
         <v>364</v>
       </c>
       <c r="B39" s="96"/>
@@ -11713,41 +11713,41 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="132" t="s">
+      <c r="A43" s="123" t="s">
         <v>392</v>
       </c>
-      <c r="B43" s="132"/>
-      <c r="C43" s="132"/>
-      <c r="D43" s="132"/>
-      <c r="E43" s="132"/>
-      <c r="F43" s="132"/>
-      <c r="G43" s="132"/>
-      <c r="H43" s="132"/>
-      <c r="I43" s="132"/>
-      <c r="J43" s="132"/>
-      <c r="K43" s="132"/>
-      <c r="L43" s="132"/>
-      <c r="M43" s="133"/>
+      <c r="B43" s="123"/>
+      <c r="C43" s="123"/>
+      <c r="D43" s="123"/>
+      <c r="E43" s="123"/>
+      <c r="F43" s="123"/>
+      <c r="G43" s="123"/>
+      <c r="H43" s="123"/>
+      <c r="I43" s="123"/>
+      <c r="J43" s="123"/>
+      <c r="K43" s="123"/>
+      <c r="L43" s="123"/>
+      <c r="M43" s="124"/>
       <c r="N43" s="70" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="101" t="s">
+      <c r="A44" s="115" t="s">
         <v>393</v>
       </c>
-      <c r="B44" s="99"/>
-      <c r="C44" s="99"/>
-      <c r="D44" s="99"/>
-      <c r="E44" s="99"/>
-      <c r="F44" s="99"/>
-      <c r="G44" s="99"/>
-      <c r="H44" s="99"/>
-      <c r="I44" s="99"/>
-      <c r="J44" s="99"/>
-      <c r="K44" s="99"/>
-      <c r="L44" s="99"/>
-      <c r="M44" s="100"/>
+      <c r="B44" s="116"/>
+      <c r="C44" s="116"/>
+      <c r="D44" s="116"/>
+      <c r="E44" s="116"/>
+      <c r="F44" s="116"/>
+      <c r="G44" s="116"/>
+      <c r="H44" s="116"/>
+      <c r="I44" s="116"/>
+      <c r="J44" s="116"/>
+      <c r="K44" s="116"/>
+      <c r="L44" s="116"/>
+      <c r="M44" s="117"/>
       <c r="N44" s="70" t="s">
         <v>76</v>
       </c>
@@ -11885,7 +11885,7 @@
       </c>
     </row>
     <row r="48" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="105" t="s">
+      <c r="A48" s="95" t="s">
         <v>421</v>
       </c>
       <c r="B48" s="96"/>
@@ -12037,21 +12037,21 @@
       </c>
     </row>
     <row r="52" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="134" t="s">
+      <c r="A52" s="111" t="s">
         <v>441</v>
       </c>
-      <c r="B52" s="134"/>
-      <c r="C52" s="134"/>
-      <c r="D52" s="134"/>
-      <c r="E52" s="134"/>
-      <c r="F52" s="134"/>
-      <c r="G52" s="134"/>
-      <c r="H52" s="134"/>
-      <c r="I52" s="134"/>
-      <c r="J52" s="134"/>
-      <c r="K52" s="134"/>
-      <c r="L52" s="134"/>
-      <c r="M52" s="135"/>
+      <c r="B52" s="111"/>
+      <c r="C52" s="111"/>
+      <c r="D52" s="111"/>
+      <c r="E52" s="111"/>
+      <c r="F52" s="111"/>
+      <c r="G52" s="111"/>
+      <c r="H52" s="111"/>
+      <c r="I52" s="111"/>
+      <c r="J52" s="111"/>
+      <c r="K52" s="111"/>
+      <c r="L52" s="111"/>
+      <c r="M52" s="112"/>
       <c r="N52" s="70" t="s">
         <v>76</v>
       </c>
@@ -12233,21 +12233,21 @@
       </c>
     </row>
     <row r="57" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="108" t="s">
+      <c r="A57" s="119" t="s">
         <v>442</v>
       </c>
-      <c r="B57" s="99"/>
-      <c r="C57" s="99"/>
-      <c r="D57" s="99"/>
-      <c r="E57" s="99"/>
-      <c r="F57" s="99"/>
-      <c r="G57" s="99"/>
-      <c r="H57" s="99"/>
-      <c r="I57" s="99"/>
-      <c r="J57" s="99"/>
-      <c r="K57" s="99"/>
-      <c r="L57" s="99"/>
-      <c r="M57" s="100"/>
+      <c r="B57" s="116"/>
+      <c r="C57" s="116"/>
+      <c r="D57" s="116"/>
+      <c r="E57" s="116"/>
+      <c r="F57" s="116"/>
+      <c r="G57" s="116"/>
+      <c r="H57" s="116"/>
+      <c r="I57" s="116"/>
+      <c r="J57" s="116"/>
+      <c r="K57" s="116"/>
+      <c r="L57" s="116"/>
+      <c r="M57" s="117"/>
       <c r="N57" s="70" t="s">
         <v>76</v>
       </c>
@@ -12385,21 +12385,21 @@
       </c>
     </row>
     <row r="61" spans="1:14" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="136" t="s">
+      <c r="A61" s="125" t="s">
         <v>500</v>
       </c>
-      <c r="B61" s="136"/>
-      <c r="C61" s="136"/>
-      <c r="D61" s="136"/>
-      <c r="E61" s="136"/>
-      <c r="F61" s="136"/>
-      <c r="G61" s="136"/>
-      <c r="H61" s="136"/>
-      <c r="I61" s="136"/>
-      <c r="J61" s="136"/>
-      <c r="K61" s="136"/>
-      <c r="L61" s="136"/>
-      <c r="M61" s="137"/>
+      <c r="B61" s="125"/>
+      <c r="C61" s="125"/>
+      <c r="D61" s="125"/>
+      <c r="E61" s="125"/>
+      <c r="F61" s="125"/>
+      <c r="G61" s="125"/>
+      <c r="H61" s="125"/>
+      <c r="I61" s="125"/>
+      <c r="J61" s="125"/>
+      <c r="K61" s="125"/>
+      <c r="L61" s="125"/>
+      <c r="M61" s="126"/>
       <c r="N61" s="70" t="s">
         <v>76</v>
       </c>
@@ -12801,7 +12801,7 @@
       </c>
     </row>
     <row r="71" spans="1:14" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="107" t="s">
+      <c r="A71" s="99" t="s">
         <v>577</v>
       </c>
       <c r="B71" s="96"/>
@@ -12953,21 +12953,21 @@
       </c>
     </row>
     <row r="75" spans="1:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="138" t="s">
+      <c r="A75" s="109" t="s">
         <v>604</v>
       </c>
-      <c r="B75" s="138"/>
-      <c r="C75" s="138"/>
-      <c r="D75" s="138"/>
-      <c r="E75" s="138"/>
-      <c r="F75" s="138"/>
-      <c r="G75" s="138"/>
-      <c r="H75" s="138"/>
-      <c r="I75" s="138"/>
-      <c r="J75" s="138"/>
-      <c r="K75" s="138"/>
-      <c r="L75" s="138"/>
-      <c r="M75" s="139"/>
+      <c r="B75" s="109"/>
+      <c r="C75" s="109"/>
+      <c r="D75" s="109"/>
+      <c r="E75" s="109"/>
+      <c r="F75" s="109"/>
+      <c r="G75" s="109"/>
+      <c r="H75" s="109"/>
+      <c r="I75" s="109"/>
+      <c r="J75" s="109"/>
+      <c r="K75" s="109"/>
+      <c r="L75" s="109"/>
+      <c r="M75" s="110"/>
       <c r="N75" s="70" t="s">
         <v>76</v>
       </c>
@@ -13105,21 +13105,21 @@
       </c>
     </row>
     <row r="79" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="134" t="s">
+      <c r="A79" s="111" t="s">
         <v>633</v>
       </c>
-      <c r="B79" s="134"/>
-      <c r="C79" s="134"/>
-      <c r="D79" s="134"/>
-      <c r="E79" s="134"/>
-      <c r="F79" s="134"/>
-      <c r="G79" s="134"/>
-      <c r="H79" s="134"/>
-      <c r="I79" s="134"/>
-      <c r="J79" s="134"/>
-      <c r="K79" s="134"/>
-      <c r="L79" s="134"/>
-      <c r="M79" s="135"/>
+      <c r="B79" s="111"/>
+      <c r="C79" s="111"/>
+      <c r="D79" s="111"/>
+      <c r="E79" s="111"/>
+      <c r="F79" s="111"/>
+      <c r="G79" s="111"/>
+      <c r="H79" s="111"/>
+      <c r="I79" s="111"/>
+      <c r="J79" s="111"/>
+      <c r="K79" s="111"/>
+      <c r="L79" s="111"/>
+      <c r="M79" s="112"/>
       <c r="N79" s="70" t="s">
         <v>76</v>
       </c>
@@ -13213,21 +13213,21 @@
       </c>
     </row>
     <row r="82" spans="1:14" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="140" t="s">
+      <c r="A82" s="113" t="s">
         <v>652</v>
       </c>
-      <c r="B82" s="140"/>
-      <c r="C82" s="140"/>
-      <c r="D82" s="140"/>
-      <c r="E82" s="140"/>
-      <c r="F82" s="140"/>
-      <c r="G82" s="140"/>
-      <c r="H82" s="140"/>
-      <c r="I82" s="140"/>
-      <c r="J82" s="140"/>
-      <c r="K82" s="140"/>
-      <c r="L82" s="140"/>
-      <c r="M82" s="141"/>
+      <c r="B82" s="113"/>
+      <c r="C82" s="113"/>
+      <c r="D82" s="113"/>
+      <c r="E82" s="113"/>
+      <c r="F82" s="113"/>
+      <c r="G82" s="113"/>
+      <c r="H82" s="113"/>
+      <c r="I82" s="113"/>
+      <c r="J82" s="113"/>
+      <c r="K82" s="113"/>
+      <c r="L82" s="113"/>
+      <c r="M82" s="114"/>
       <c r="N82" s="70" t="s">
         <v>76</v>
       </c>
@@ -13577,7 +13577,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="97" t="s">
         <v>712</v>
       </c>
       <c r="B1" s="96"/>
@@ -13591,7 +13591,7 @@
       <c r="J1" s="96"/>
     </row>
     <row r="2" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="104" t="s">
         <v>713</v>
       </c>
       <c r="B2" s="96"/>
@@ -13640,7 +13640,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="104" t="s">
+      <c r="A4" s="102" t="s">
         <v>75</v>
       </c>
       <c r="B4" s="96"/>
@@ -14346,7 +14346,7 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="114" t="s">
+      <c r="A28" s="105" t="s">
         <v>309</v>
       </c>
       <c r="B28" s="96"/>
@@ -14559,7 +14559,7 @@
       </c>
     </row>
     <row r="35" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="106" t="s">
+      <c r="A35" s="101" t="s">
         <v>364</v>
       </c>
       <c r="B35" s="96"/>
@@ -14661,7 +14661,7 @@
       </c>
     </row>
     <row r="39" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="111" t="s">
+      <c r="A39" s="100" t="s">
         <v>392</v>
       </c>
       <c r="B39" s="96"/>
@@ -14794,7 +14794,7 @@
       </c>
     </row>
     <row r="44" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="105" t="s">
+      <c r="A44" s="95" t="s">
         <v>421</v>
       </c>
       <c r="B44" s="96"/>
@@ -14896,7 +14896,7 @@
       </c>
     </row>
     <row r="48" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="112" t="s">
+      <c r="A48" s="103" t="s">
         <v>441</v>
       </c>
       <c r="B48" s="96"/>
@@ -15143,7 +15143,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="107" t="s">
+      <c r="A57" s="99" t="s">
         <v>500</v>
       </c>
       <c r="B57" s="96"/>
@@ -15397,7 +15397,7 @@
       </c>
     </row>
     <row r="67" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="107" t="s">
+      <c r="A67" s="99" t="s">
         <v>577</v>
       </c>
       <c r="B67" s="96"/>
@@ -15524,7 +15524,7 @@
       </c>
     </row>
     <row r="72" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="105" t="s">
+      <c r="A72" s="95" t="s">
         <v>604</v>
       </c>
       <c r="B72" s="96"/>
@@ -15626,7 +15626,7 @@
       </c>
     </row>
     <row r="76" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="112" t="s">
+      <c r="A76" s="103" t="s">
         <v>633</v>
       </c>
       <c r="B76" s="96"/>
@@ -15695,7 +15695,7 @@
       </c>
     </row>
     <row r="79" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="110" t="s">
+      <c r="A79" s="98" t="s">
         <v>652</v>
       </c>
       <c r="B79" s="96"/>
@@ -16152,7 +16152,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="97" t="s">
         <v>841</v>
       </c>
       <c r="B1" s="96"/>
@@ -16167,7 +16167,7 @@
       <c r="K1" s="96"/>
     </row>
     <row r="2" spans="1:12" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="104" t="s">
         <v>842</v>
       </c>
       <c r="B2" s="96"/>
@@ -16220,7 +16220,7 @@
       </c>
     </row>
     <row r="4" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="104" t="s">
+      <c r="A4" s="102" t="s">
         <v>75</v>
       </c>
       <c r="B4" s="96"/>
@@ -17109,7 +17109,7 @@
       </c>
     </row>
     <row r="28" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="114" t="s">
+      <c r="A28" s="105" t="s">
         <v>309</v>
       </c>
       <c r="B28" s="96"/>
@@ -17352,7 +17352,7 @@
       </c>
     </row>
     <row r="35" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="106" t="s">
+      <c r="A35" s="101" t="s">
         <v>364</v>
       </c>
       <c r="B35" s="96"/>
@@ -17481,7 +17481,7 @@
       </c>
     </row>
     <row r="39" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="111" t="s">
+      <c r="A39" s="100" t="s">
         <v>392</v>
       </c>
       <c r="B39" s="96"/>
@@ -17648,7 +17648,7 @@
       </c>
     </row>
     <row r="44" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="105" t="s">
+      <c r="A44" s="95" t="s">
         <v>421</v>
       </c>
       <c r="B44" s="96"/>
@@ -17777,7 +17777,7 @@
       </c>
     </row>
     <row r="48" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="112" t="s">
+      <c r="A48" s="103" t="s">
         <v>441</v>
       </c>
       <c r="B48" s="96"/>
@@ -18096,7 +18096,7 @@
       </c>
     </row>
     <row r="57" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="107" t="s">
+      <c r="A57" s="99" t="s">
         <v>500</v>
       </c>
       <c r="B57" s="96"/>
@@ -18453,7 +18453,7 @@
       </c>
     </row>
     <row r="67" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="107" t="s">
+      <c r="A67" s="99" t="s">
         <v>577</v>
       </c>
       <c r="B67" s="96"/>
@@ -18620,7 +18620,7 @@
       </c>
     </row>
     <row r="72" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="105" t="s">
+      <c r="A72" s="95" t="s">
         <v>604</v>
       </c>
       <c r="B72" s="96"/>
@@ -18749,7 +18749,7 @@
       </c>
     </row>
     <row r="76" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="112" t="s">
+      <c r="A76" s="103" t="s">
         <v>633</v>
       </c>
       <c r="B76" s="96"/>
@@ -18840,7 +18840,7 @@
       </c>
     </row>
     <row r="79" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="110" t="s">
+      <c r="A79" s="98" t="s">
         <v>652</v>
       </c>
       <c r="B79" s="96"/>
@@ -19350,6 +19350,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A67:K67"/>
+    <mergeCell ref="A35:K35"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A48:K48"/>
     <mergeCell ref="A79:K79"/>
     <mergeCell ref="A39:K39"/>
     <mergeCell ref="A72:K72"/>
@@ -19358,11 +19363,6 @@
     <mergeCell ref="A28:K28"/>
     <mergeCell ref="A76:K76"/>
     <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A67:K67"/>
-    <mergeCell ref="A35:K35"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A48:K48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19388,7 +19388,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
+      <c r="A1" s="97" t="s">
         <v>1157</v>
       </c>
       <c r="B1" s="96"/>
@@ -19408,7 +19408,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="115" t="s">
+      <c r="A2" s="127" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -20245,13 +20245,13 @@
         <v>1279</v>
       </c>
       <c r="H18" s="6" t="s">
+        <v>1860</v>
+      </c>
+      <c r="I18" s="6" t="s">
         <v>1280</v>
       </c>
-      <c r="I18" s="6" t="s">
+      <c r="J18" s="6" t="s">
         <v>1281</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>1282</v>
       </c>
       <c r="K18" s="6" t="s">
         <v>864</v>
@@ -20269,7 +20269,7 @@
         <v>82</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="Q18" s="70" t="s">
         <v>76</v>
@@ -20277,7 +20277,7 @@
     </row>
     <row r="19" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="81" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="B19" s="8" t="s">
         <v>34</v>
@@ -20289,22 +20289,22 @@
         <v>291</v>
       </c>
       <c r="E19" s="8" t="s">
+        <v>1284</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>1285</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="G19" s="8" t="s">
         <v>1286</v>
       </c>
-      <c r="G19" s="8" t="s">
+      <c r="H19" s="8" t="s">
         <v>1287</v>
       </c>
-      <c r="H19" s="8" t="s">
+      <c r="I19" s="8" t="s">
         <v>1288</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="J19" s="8" t="s">
         <v>1289</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>1290</v>
       </c>
       <c r="K19" s="8" t="s">
         <v>864</v>
@@ -20322,7 +20322,7 @@
         <v>82</v>
       </c>
       <c r="P19" s="8" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="Q19" s="70" t="s">
         <v>76</v>
@@ -20330,7 +20330,7 @@
     </row>
     <row r="20" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="80" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>34</v>
@@ -20342,22 +20342,22 @@
         <v>300</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>1292</v>
+      </c>
+      <c r="F20" s="6" t="s">
         <v>1293</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="G20" s="6" t="s">
         <v>1294</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="H20" s="6" t="s">
         <v>1295</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="I20" s="6" t="s">
         <v>1296</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="J20" s="6" t="s">
         <v>1297</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>1298</v>
       </c>
       <c r="K20" s="6" t="s">
         <v>900</v>
@@ -20375,7 +20375,7 @@
         <v>82</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="Q20" s="70" t="s">
         <v>76</v>
@@ -20410,8 +20410,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1300</v>
+      <c r="A1" s="97" t="s">
+        <v>1299</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -20430,7 +20430,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="116" t="s">
+      <c r="A2" s="128" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -20504,7 +20504,7 @@
     </row>
     <row r="4" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="49" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>37</v>
@@ -20516,22 +20516,22 @@
         <v>312</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>1301</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>1302</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>1303</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>1304</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>1305</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>1306</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>1307</v>
       </c>
       <c r="K4" s="45" t="s">
         <v>864</v>
@@ -20549,7 +20549,7 @@
         <v>82</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="Q4" s="70" t="s">
         <v>76</v>
@@ -20557,7 +20557,7 @@
     </row>
     <row r="5" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="50" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>37</v>
@@ -20569,22 +20569,22 @@
         <v>320</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>1309</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>1310</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>1311</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>1312</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>1313</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>1314</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>1315</v>
       </c>
       <c r="K5" s="47" t="s">
         <v>864</v>
@@ -20602,7 +20602,7 @@
         <v>82</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="Q5" s="70" t="s">
         <v>76</v>
@@ -20610,7 +20610,7 @@
     </row>
     <row r="6" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="49" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>37</v>
@@ -20622,22 +20622,22 @@
         <v>328</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>1317</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>1318</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>1319</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>1320</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>1321</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>1322</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>1323</v>
       </c>
       <c r="K6" s="45" t="s">
         <v>900</v>
@@ -20655,7 +20655,7 @@
         <v>82</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="Q6" s="70" t="s">
         <v>76</v>
@@ -20663,7 +20663,7 @@
     </row>
     <row r="7" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="50" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>37</v>
@@ -20675,22 +20675,22 @@
         <v>762</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>1325</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>1326</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>1327</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>1328</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>1329</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>1330</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>1331</v>
       </c>
       <c r="K7" s="47" t="s">
         <v>875</v>
@@ -20708,7 +20708,7 @@
         <v>82</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="Q7" s="70" t="s">
         <v>76</v>
@@ -20716,7 +20716,7 @@
     </row>
     <row r="8" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="49" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>37</v>
@@ -20728,22 +20728,22 @@
         <v>337</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>1333</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>1334</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>1335</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>1336</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>1337</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>1338</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>1339</v>
       </c>
       <c r="K8" s="45" t="s">
         <v>880</v>
@@ -20761,7 +20761,7 @@
         <v>109</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="Q8" s="70" t="s">
         <v>76</v>
@@ -20769,7 +20769,7 @@
     </row>
     <row r="9" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="50" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>37</v>
@@ -20781,22 +20781,22 @@
         <v>346</v>
       </c>
       <c r="E9" s="8" t="s">
+        <v>1341</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>1342</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>1343</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>765</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>1343</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>1344</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>1345</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>1346</v>
       </c>
       <c r="K9" s="47" t="s">
         <v>875</v>
@@ -20814,7 +20814,7 @@
         <v>109</v>
       </c>
       <c r="P9" s="8" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="Q9" s="70" t="s">
         <v>76</v>
@@ -20822,7 +20822,7 @@
     </row>
     <row r="10" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="82" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>37</v>
@@ -20834,22 +20834,22 @@
         <v>355</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>1348</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>1349</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>1350</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>1351</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>1352</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>1353</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>1354</v>
       </c>
       <c r="K10" s="6" t="s">
         <v>875</v>
@@ -20867,7 +20867,7 @@
         <v>109</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="Q10" s="70" t="s">
         <v>76</v>
@@ -20902,8 +20902,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1356</v>
+      <c r="A1" s="97" t="s">
+        <v>1355</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -20922,7 +20922,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="117" t="s">
+      <c r="A2" s="129" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -20996,7 +20996,7 @@
     </row>
     <row r="4" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="52" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>40</v>
@@ -21008,22 +21008,22 @@
         <v>366</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>1357</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>1358</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>1359</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>765</v>
       </c>
       <c r="H4" s="6" t="s">
+        <v>1359</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>1360</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>1361</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>1362</v>
       </c>
       <c r="K4" s="45" t="s">
         <v>880</v>
@@ -21041,7 +21041,7 @@
         <v>109</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="Q4" s="70" t="s">
         <v>76</v>
@@ -21049,34 +21049,34 @@
     </row>
     <row r="5" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="53" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>374</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>767</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>1365</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>1366</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>1367</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>1368</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>1369</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>1370</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>1371</v>
       </c>
       <c r="K5" s="47" t="s">
         <v>875</v>
@@ -21094,7 +21094,7 @@
         <v>109</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
       <c r="Q5" s="70" t="s">
         <v>76</v>
@@ -21102,7 +21102,7 @@
     </row>
     <row r="6" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="52" t="s">
-        <v>1373</v>
+        <v>1372</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>40</v>
@@ -21114,22 +21114,22 @@
         <v>384</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>1373</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>1374</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>1375</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>1376</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>1377</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>1378</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>1379</v>
       </c>
       <c r="K6" s="45" t="s">
         <v>900</v>
@@ -21147,7 +21147,7 @@
         <v>109</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="Q6" s="70" t="s">
         <v>76</v>
@@ -21155,7 +21155,7 @@
     </row>
     <row r="7" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="53" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>46</v>
@@ -21167,22 +21167,22 @@
         <v>432</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>1381</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>1382</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>1383</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>778</v>
       </c>
       <c r="H7" s="8" t="s">
+        <v>1383</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>1384</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>1385</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>1386</v>
       </c>
       <c r="K7" s="47" t="s">
         <v>880</v>
@@ -21200,7 +21200,7 @@
         <v>109</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="Q7" s="70" t="s">
         <v>76</v>
@@ -21208,34 +21208,34 @@
     </row>
     <row r="8" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="52" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>40</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>346</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>1389</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>1390</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>1391</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>765</v>
       </c>
       <c r="H8" s="6" t="s">
+        <v>1391</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>1392</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>1393</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>1394</v>
       </c>
       <c r="K8" s="45" t="s">
         <v>875</v>
@@ -21253,7 +21253,7 @@
         <v>109</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>1395</v>
+        <v>1394</v>
       </c>
       <c r="Q8" s="70" t="s">
         <v>76</v>
@@ -21288,8 +21288,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1396</v>
+      <c r="A1" s="97" t="s">
+        <v>1395</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -21308,7 +21308,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="118" t="s">
+      <c r="A2" s="130" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -21382,7 +21382,7 @@
     </row>
     <row r="4" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="55" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>43</v>
@@ -21391,25 +21391,25 @@
         <v>394</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>1397</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>1398</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>1399</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>1400</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>771</v>
       </c>
       <c r="H4" s="6" t="s">
+        <v>1400</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>1401</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>1402</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>1403</v>
       </c>
       <c r="K4" s="45" t="s">
         <v>875</v>
@@ -21427,7 +21427,7 @@
         <v>82</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="Q4" s="70" t="s">
         <v>76</v>
@@ -21435,7 +21435,7 @@
     </row>
     <row r="5" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="56" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>43</v>
@@ -21447,22 +21447,22 @@
         <v>395</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>1405</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>1406</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="8" t="s">
         <v>1407</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>1408</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="8" t="s">
         <v>1409</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="J5" s="8" t="s">
         <v>1410</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>1411</v>
       </c>
       <c r="K5" s="47" t="s">
         <v>864</v>
@@ -21480,7 +21480,7 @@
         <v>82</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>1412</v>
+        <v>1411</v>
       </c>
       <c r="Q5" s="70" t="s">
         <v>76</v>
@@ -21488,7 +21488,7 @@
     </row>
     <row r="6" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="55" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>43</v>
@@ -21500,22 +21500,22 @@
         <v>404</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>1413</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>1414</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>1415</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>773</v>
       </c>
       <c r="H6" s="6" t="s">
+        <v>1415</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>1416</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>1417</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>1418</v>
       </c>
       <c r="K6" s="45" t="s">
         <v>880</v>
@@ -21533,7 +21533,7 @@
         <v>109</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="Q6" s="70" t="s">
         <v>76</v>
@@ -21541,7 +21541,7 @@
     </row>
     <row r="7" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="56" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>43</v>
@@ -21553,22 +21553,22 @@
         <v>413</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>1420</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>1421</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>1422</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>775</v>
       </c>
       <c r="H7" s="8" t="s">
+        <v>1422</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>1423</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>1424</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>1425</v>
       </c>
       <c r="K7" s="47" t="s">
         <v>854</v>
@@ -21586,7 +21586,7 @@
         <v>82</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="Q7" s="70" t="s">
         <v>76</v>
@@ -21621,8 +21621,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="102" t="s">
-        <v>1427</v>
+      <c r="A1" s="97" t="s">
+        <v>1426</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -21641,7 +21641,7 @@
       <c r="P1" s="96"/>
     </row>
     <row r="2" spans="1:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="119" t="s">
+      <c r="A2" s="131" t="s">
         <v>1158</v>
       </c>
       <c r="B2" s="96"/>
@@ -21715,7 +21715,7 @@
     </row>
     <row r="4" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="58" t="s">
-        <v>1428</v>
+        <v>1427</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>46</v>
@@ -21727,22 +21727,22 @@
         <v>424</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>1428</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>1429</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>1430</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>1431</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>1432</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>1433</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>1434</v>
       </c>
       <c r="K4" s="45" t="s">
         <v>900</v>
@@ -21760,7 +21760,7 @@
         <v>82</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1435</v>
+        <v>1434</v>
       </c>
       <c r="Q4" s="70" t="s">
         <v>76</v>
@@ -21768,7 +21768,7 @@
     </row>
     <row r="5" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="59" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>46</v>
@@ -21780,22 +21780,22 @@
         <v>432</v>
       </c>
       <c r="E5" s="8" t="s">
+        <v>1436</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>1437</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>1438</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>778</v>
       </c>
       <c r="H5" s="8" t="s">
+        <v>1438</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>1439</v>
       </c>
-      <c r="I5" s="8" t="s">
-        <v>1440</v>
-      </c>
       <c r="J5" s="8" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="K5" s="47" t="s">
         <v>880</v>
@@ -21813,7 +21813,7 @@
         <v>109</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="Q5" s="70" t="s">
         <v>76</v>
@@ -21821,7 +21821,7 @@
     </row>
     <row r="6" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="58" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>46</v>
@@ -21833,22 +21833,22 @@
         <v>211</v>
       </c>
       <c r="E6" s="6" t="s">
+        <v>1441</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>1442</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>1443</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>1444</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>1445</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>1446</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>1447</v>
       </c>
       <c r="K6" s="45" t="s">
         <v>900</v>
@@ -21866,7 +21866,7 @@
         <v>82</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="Q6" s="71" t="s">
         <v>227</v>
@@ -21874,7 +21874,7 @@
     </row>
     <row r="7" spans="1:17" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="59" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>46</v>
@@ -21886,22 +21886,22 @@
         <v>750</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>1449</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>1450</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>1451</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>1452</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>1453</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>1454</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>1455</v>
       </c>
       <c r="K7" s="47" t="s">
         <v>880</v>
@@ -21919,7 +21919,7 @@
         <v>109</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
       <c r="Q7" s="71" t="s">
         <v>227</v>

</xml_diff>